<commit_message>
Quitar el panel congelado de la lista de chequeo
La cabecera del instrumento —logo, datos del aprendiz, indicadores y
cabecera de tabla— mide mas de 400 px. Al inmovilizarla, esas catorce
filas se quedaban fijas y ocupaban casi toda la pantalla, dejando una
franja de desplazamiento tan estrecha que las capturas, que miden entre
200 y 400 puntos de alto, no se llegaban a ver enteras. Parecia que no
estuvieran puestas.

Ahora la hoja se desplaza entera. Para imprimir sigue repitiendose la
fila de cabecera en cada pagina, que es donde esa ayuda si suma.

Se rellena tambien el documento de identidad, como texto y no como
numero: es un identificador, no una cantidad.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidencias/Lista_Chequeo_Cuarto_Avance_AutoPrime.xlsx
+++ b/evidencias/Lista_Chequeo_Cuarto_Avance_AutoPrime.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
   <si>
     <t>SENA - REGIONAL ANTIOQUIA</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t>Documento de Identidad:</t>
+  </si>
+  <si>
+    <t>1038928023</t>
   </si>
   <si>
     <t>Ficha de Caracterización:</t>
@@ -2087,47 +2090,49 @@
         <v>8</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="C7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="D7" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="22" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="22" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20" customHeight="1">
       <c r="A10" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -2136,13 +2141,13 @@
     </row>
     <row r="11" spans="1:5" ht="26" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11" s="6">
         <v>26</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="6">
         <v>26</v>
@@ -2154,22 +2159,22 @@
     </row>
     <row r="12" spans="1:5" ht="22" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="20" customHeight="1">
       <c r="A13" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -2178,430 +2183,430 @@
     </row>
     <row r="14" spans="1:5" ht="34" customHeight="1">
       <c r="A14" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="213.544" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="163.418" customHeight="1">
       <c r="A16" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D16" s="21"/>
       <c r="E16" s="17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="117.848" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="112.785" customHeight="1">
       <c r="A18" s="18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D18" s="21"/>
       <c r="E18" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="143.165" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="213.544" customHeight="1">
       <c r="A20" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="21"/>
       <c r="E20" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="213.544" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D21" s="16"/>
       <c r="E21" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="102.658" customHeight="1">
       <c r="A22" s="18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" s="21"/>
       <c r="E22" s="17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="213.544" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="213.544" customHeight="1">
       <c r="A24" s="18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D24" s="21"/>
       <c r="E24" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="148.228" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D25" s="16"/>
       <c r="E25" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="102.658" customHeight="1">
       <c r="A26" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D26" s="21"/>
       <c r="E26" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="133.038" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="213.544" customHeight="1">
       <c r="A28" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D28" s="21"/>
       <c r="E28" s="17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="213.544" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="213.544" customHeight="1">
       <c r="A30" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D30" s="21"/>
       <c r="E30" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="213.544" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="213.544" customHeight="1">
       <c r="A32" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D32" s="21"/>
       <c r="E32" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="213.544" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D33" s="16"/>
       <c r="E33" s="17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="213.544" customHeight="1">
       <c r="A34" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D34" s="21"/>
       <c r="E34" s="17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="213.544" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="102.658" customHeight="1">
       <c r="A36" s="18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D36" s="21"/>
       <c r="E36" s="17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="264.684" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="17" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="213.544" customHeight="1">
       <c r="A38" s="18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D38" s="21"/>
       <c r="E38" s="17" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="213.544" customHeight="1">
       <c r="A39" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D39" s="16"/>
       <c r="E39" s="17" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="234.304" customHeight="1">
       <c r="A40" s="18" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D40" s="21"/>
       <c r="E40" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="24" customHeight="1">
       <c r="A41" s="22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B41" s="22"/>
       <c r="C41" s="22"/>
       <c r="D41" s="23" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E41" s="23"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="24" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="24" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>